<commit_message>
Added support for Discover Bank
</commit_message>
<xml_diff>
--- a/examples/discover-card.xlsx
+++ b/examples/discover-card.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\eschrock\bugjet\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D1A20C-D2FC-41A6-B5BD-DD3D7D9D9284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CFA8A58-A478-436B-BA04-74DB5FCC30E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0855052D-DBE2-40F6-8B44-10FDCBDF92BC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
   <si>
     <t>Trans. Date</t>
   </si>
@@ -65,10 +65,7 @@
     <t>C</t>
   </si>
   <si>
-    <t>INTERNET PAYMENT - THANK YOU</t>
-  </si>
-  <si>
-    <t>Payments and Credits</t>
+    <t>E</t>
   </si>
 </sst>
 </file>
@@ -552,8 +549,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -916,7 +912,7 @@
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="55.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -939,88 +935,88 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45302</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>45302</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2">
         <v>21.39</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45302</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>45302</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3">
         <v>40.71</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45303</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>45303</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4">
         <v>21.98</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45304</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>45304</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5">
         <v>12.51</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45304</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>45304</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6">
         <v>-412.73</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>10</v>
+      <c r="E6" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>